<commit_message>
Implementation of data driven testing using Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/PIMData.xlsx
+++ b/src/test/resources/testdata/PIMData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ScriptX_Project\ScriptX_OrangeHRM\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5319844-7EA5-487F-A045-724CE798C68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B8FC5EB-7CE1-44DF-8C63-A7512119D6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2158354C-DBF5-4CF8-89A0-7207B40B3FD2}"/>
   </bookViews>
@@ -34,12 +34,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>employeeName</t>
   </si>
   <si>
-    <t>jagadee</t>
+    <t>employeeId</t>
+  </si>
+  <si>
+    <t>Kumaar</t>
+  </si>
+  <si>
+    <t>Akashh</t>
+  </si>
+  <si>
+    <t>jagadeep</t>
   </si>
 </sst>
 </file>
@@ -391,20 +400,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10B53E58-A9E5-4C90-A6E0-1F6F813AD7E5}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>9011</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>9011</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>1223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>